<commit_message>
new files for june 2026
</commit_message>
<xml_diff>
--- a/web-tool-table-process/materials/CancerSiteTable_samp.xlsx
+++ b/web-tool-table-process/materials/CancerSiteTable_samp.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Westat.com\dfs\SEER\Geospatial Activities\SEER_Zone_Design\~Specific Registry Zoning\Louisiana\ZoneRateCalcs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\westat.com\dfs\SEER\Geospatial Activities\SEER_Zone_Design\Step_3c_WebToolTables\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CC07905-3CA3-4CB7-850C-E9BAB357082E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18870" windowHeight="9630" tabRatio="659"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="659" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEER_Stat" sheetId="1" r:id="rId1"/>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="75">
   <si>
     <t>All Sites</t>
   </si>
@@ -157,54 +158,6 @@
     <t>All Cancer Sites</t>
   </si>
   <si>
-    <t>Prostate Cancer</t>
-  </si>
-  <si>
-    <t>Lung Cancer</t>
-  </si>
-  <si>
-    <t>Breast Cancer</t>
-  </si>
-  <si>
-    <t>Colonrectal Cancer</t>
-  </si>
-  <si>
-    <t>Kidney and Renal Pelvis Cancer</t>
-  </si>
-  <si>
-    <t>Urinary Bladder Cancer</t>
-  </si>
-  <si>
-    <t>Pancreatic Cancer</t>
-  </si>
-  <si>
-    <t>Oral Cavity and Pharynx Cancer</t>
-  </si>
-  <si>
-    <t>Thyroid Cancer</t>
-  </si>
-  <si>
-    <t>Uterine Corpus Cancer</t>
-  </si>
-  <si>
-    <t>Liver Cancer</t>
-  </si>
-  <si>
-    <t>Stomach Cancer</t>
-  </si>
-  <si>
-    <t>Brain Cancer</t>
-  </si>
-  <si>
-    <t>Larynx Cancer</t>
-  </si>
-  <si>
-    <t>Ovarian Cancer</t>
-  </si>
-  <si>
-    <t>Esophagian Cancer</t>
-  </si>
-  <si>
     <t>Esoph</t>
   </si>
   <si>
@@ -299,12 +252,15 @@
   </si>
   <si>
     <t>Non-Hispanic Black</t>
+  </si>
+  <si>
+    <t>Female Breast</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -346,7 +302,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -362,6 +318,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -626,7 +586,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -642,10 +602,10 @@
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -661,10 +621,10 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -683,7 +643,7 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -763,10 +723,10 @@
         <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -817,12 +777,12 @@
         <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
         <v>16</v>
@@ -833,10 +793,10 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -855,7 +815,7 @@
         <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -885,29 +845,29 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>41</v>
       </c>
     </row>
@@ -915,47 +875,47 @@
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>42</v>
+      <c r="B3" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
-        <v>43</v>
+      <c r="B4" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
-        <v>44</v>
+      <c r="B5" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="s">
-        <v>45</v>
+      <c r="B6" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
-        <v>46</v>
+      <c r="B7" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -963,15 +923,15 @@
       <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" t="s">
-        <v>47</v>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -979,15 +939,15 @@
       <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="B11" t="s">
-        <v>48</v>
+      <c r="B11" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>35</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -995,47 +955,47 @@
       <c r="A13" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
-        <v>49</v>
+      <c r="B13" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
-      <c r="B14" t="s">
-        <v>50</v>
+      <c r="B14" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>36</v>
       </c>
-      <c r="B15" t="s">
-        <v>51</v>
+      <c r="B15" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>28</v>
       </c>
-      <c r="B16" t="s">
-        <v>52</v>
+      <c r="B16" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>12</v>
       </c>
-      <c r="B17" t="s">
-        <v>53</v>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1043,47 +1003,47 @@
       <c r="A19" t="s">
         <v>29</v>
       </c>
-      <c r="B19" t="s">
-        <v>54</v>
+      <c r="B19" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>15</v>
       </c>
-      <c r="B20" t="s">
-        <v>55</v>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>30</v>
       </c>
-      <c r="B21" t="s">
-        <v>56</v>
+      <c r="B21" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" t="s">
-        <v>57</v>
+        <v>42</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>31</v>
       </c>
-      <c r="B23" t="s">
-        <v>72</v>
+      <c r="B23" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>38</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1091,7 +1051,7 @@
       <c r="A25" t="s">
         <v>32</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1099,7 +1059,7 @@
       <c r="A26" t="s">
         <v>40</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1107,7 +1067,7 @@
       <c r="A27" t="s">
         <v>39</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1122,7 +1082,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1134,34 +1094,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1175,7 +1135,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1187,10 +1147,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1198,7 +1158,7 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1206,7 +1166,7 @@
         <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1214,7 +1174,7 @@
         <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1222,15 +1182,15 @@
         <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1238,7 +1198,7 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1252,7 +1212,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1264,34 +1224,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1305,7 +1265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1317,55 +1277,55 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>